<commit_message>
feat: update import and calculation logic to remove PCD as a separate type and adjust related functionalities
</commit_message>
<xml_diff>
--- a/app/public/modelos/modelo-quantidade.xlsx
+++ b/app/public/modelos/modelo-quantidade.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,7 +427,7 @@
         <v>CLT</v>
       </c>
       <c r="D2">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -472,10 +472,10 @@
         <v>11.111.111/0001-11</v>
       </c>
       <c r="B5" t="str">
-        <v>411010</v>
+        <v>411005</v>
       </c>
       <c r="C5" t="str">
-        <v>PCD</v>
+        <v>APRENDIZ</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -486,16 +486,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>11.111.111/0001-11</v>
+        <v>11.111.111/0002-22</v>
       </c>
       <c r="B6" t="str">
-        <v>411005</v>
+        <v>411010</v>
       </c>
       <c r="C6" t="str">
-        <v>APRENDIZ</v>
+        <v>CLT</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -506,38 +506,21 @@
         <v>11.111.111/0002-22</v>
       </c>
       <c r="B7" t="str">
-        <v>411010</v>
+        <v>351305</v>
       </c>
       <c r="C7" t="str">
-        <v>CLT</v>
+        <v>ESTAGIARIO</v>
       </c>
       <c r="D7">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>11.111.111/0002-22</v>
-      </c>
-      <c r="B8" t="str">
-        <v>351305</v>
-      </c>
-      <c r="C8" t="str">
-        <v>ESTAGIARIO</v>
-      </c>
-      <c r="D8">
-        <v>2</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>